<commit_message>
optimized the code and added ART 3 & 4 to new MSF
</commit_message>
<xml_diff>
--- a/templates/New_MSF.xlsx
+++ b/templates/New_MSF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chinedu\Documents\GitHub\MSF-Calculator\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{615145CB-C3AA-4A27-9684-3C05A29C5E04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C9578D6-95F3-4EF9-B5F2-D97625869259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{2547347A-7686-4B19-BC03-747D4C25AA4C}"/>
   </bookViews>
@@ -2863,7 +2863,10 @@
       <c r="H31" s="8"/>
       <c r="I31" s="8"/>
       <c r="J31" s="8"/>
-      <c r="K31" s="4"/>
+      <c r="K31" s="22">
+        <f>SUM(C31:J31)</f>
+        <v>0</v>
+      </c>
       <c r="L31" s="58"/>
       <c r="M31" s="59"/>
     </row>
@@ -2880,7 +2883,10 @@
       <c r="H32" s="8"/>
       <c r="I32" s="8"/>
       <c r="J32" s="8"/>
-      <c r="K32" s="4"/>
+      <c r="K32" s="22">
+        <f>SUM(C32:J32)</f>
+        <v>0</v>
+      </c>
       <c r="L32" s="58"/>
       <c r="M32" s="59"/>
     </row>
@@ -2939,7 +2945,10 @@
       <c r="H35" s="70"/>
       <c r="I35" s="70"/>
       <c r="J35" s="72"/>
-      <c r="K35" s="2"/>
+      <c r="K35" s="50">
+        <f>SUM(C35:J35)</f>
+        <v>0</v>
+      </c>
       <c r="L35" s="60"/>
       <c r="M35" s="61"/>
     </row>
@@ -3025,7 +3034,10 @@
       <c r="H39" s="8"/>
       <c r="I39" s="8"/>
       <c r="J39" s="8"/>
-      <c r="K39" s="8"/>
+      <c r="K39" s="3">
+        <f>SUM(C39:J39)</f>
+        <v>0</v>
+      </c>
       <c r="L39" s="100"/>
       <c r="M39" s="59"/>
     </row>
@@ -3042,7 +3054,10 @@
       <c r="H40" s="8"/>
       <c r="I40" s="8"/>
       <c r="J40" s="8"/>
-      <c r="K40" s="8"/>
+      <c r="K40" s="3">
+        <f>SUM(C40:J40)</f>
+        <v>0</v>
+      </c>
       <c r="L40" s="100"/>
       <c r="M40" s="59"/>
     </row>
@@ -3101,7 +3116,10 @@
       <c r="H43" s="70"/>
       <c r="I43" s="70"/>
       <c r="J43" s="104"/>
-      <c r="K43" s="4"/>
+      <c r="K43" s="22">
+        <f>SUM(C43:J43)</f>
+        <v>0</v>
+      </c>
       <c r="L43" s="101"/>
       <c r="M43" s="61"/>
     </row>

</xml_diff>

<commit_message>
added ART 5 to New MSF
</commit_message>
<xml_diff>
--- a/templates/New_MSF.xlsx
+++ b/templates/New_MSF.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chinedu\Documents\GitHub\MSF-Calculator\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C9578D6-95F3-4EF9-B5F2-D97625869259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CA87D6D-560B-4957-9B2E-CDE10A5485DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{2547347A-7686-4B19-BC03-747D4C25AA4C}"/>
   </bookViews>
@@ -1344,7 +1344,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="167">
+  <cellXfs count="169">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -1496,6 +1496,9 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1843,6 +1846,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2185,21 +2191,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="52"/>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="52"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="52"/>
-      <c r="L1" s="52"/>
-      <c r="M1" s="53"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="53"/>
+      <c r="G1" s="53"/>
+      <c r="H1" s="53"/>
+      <c r="I1" s="53"/>
+      <c r="J1" s="53"/>
+      <c r="K1" s="53"/>
+      <c r="L1" s="53"/>
+      <c r="M1" s="54"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2231,10 +2237,10 @@
       <c r="K2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L2" s="54" t="s">
+      <c r="L2" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="M2" s="55"/>
+      <c r="M2" s="56"/>
     </row>
     <row r="3" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -2255,10 +2261,10 @@
         <f>SUM(C4:J5)</f>
         <v>0</v>
       </c>
-      <c r="L3" s="56" t="s">
+      <c r="L3" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="M3" s="57"/>
+      <c r="M3" s="58"/>
     </row>
     <row r="4" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2"/>
@@ -2277,8 +2283,8 @@
         <f>SUM(C4:J4)</f>
         <v>0</v>
       </c>
-      <c r="L4" s="58"/>
-      <c r="M4" s="59"/>
+      <c r="L4" s="59"/>
+      <c r="M4" s="60"/>
     </row>
     <row r="5" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
@@ -2297,27 +2303,27 @@
         <f>SUM(C5:J5)</f>
         <v>0</v>
       </c>
-      <c r="L5" s="58"/>
-      <c r="M5" s="59"/>
+      <c r="L5" s="59"/>
+      <c r="M5" s="60"/>
     </row>
     <row r="6" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="4"/>
-      <c r="C6" s="62"/>
-      <c r="D6" s="63"/>
-      <c r="E6" s="63"/>
-      <c r="F6" s="63"/>
-      <c r="G6" s="63"/>
-      <c r="H6" s="63"/>
-      <c r="I6" s="63"/>
-      <c r="J6" s="64"/>
+      <c r="C6" s="63"/>
+      <c r="D6" s="64"/>
+      <c r="E6" s="64"/>
+      <c r="F6" s="64"/>
+      <c r="G6" s="64"/>
+      <c r="H6" s="64"/>
+      <c r="I6" s="64"/>
+      <c r="J6" s="65"/>
       <c r="K6" s="9"/>
-      <c r="L6" s="58"/>
-      <c r="M6" s="59"/>
+      <c r="L6" s="59"/>
+      <c r="M6" s="60"/>
     </row>
     <row r="7" spans="1:13" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="65"/>
-      <c r="B7" s="67" t="s">
+      <c r="A7" s="66"/>
+      <c r="B7" s="68" t="s">
         <v>13</v>
       </c>
       <c r="C7" s="10" t="s">
@@ -2332,35 +2338,35 @@
       <c r="F7" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="G7" s="69" t="s">
+      <c r="G7" s="70" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="70"/>
-      <c r="I7" s="70"/>
-      <c r="J7" s="71"/>
+      <c r="H7" s="71"/>
+      <c r="I7" s="71"/>
+      <c r="J7" s="72"/>
       <c r="K7" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="L7" s="58"/>
-      <c r="M7" s="59"/>
+      <c r="L7" s="59"/>
+      <c r="M7" s="60"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="66"/>
-      <c r="B8" s="68"/>
+      <c r="A8" s="67"/>
+      <c r="B8" s="69"/>
       <c r="C8" s="1"/>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="69"/>
-      <c r="H8" s="70"/>
-      <c r="I8" s="70"/>
-      <c r="J8" s="72"/>
+      <c r="G8" s="70"/>
+      <c r="H8" s="71"/>
+      <c r="I8" s="71"/>
+      <c r="J8" s="73"/>
       <c r="K8" s="50">
         <f>SUM(C8:J8)</f>
         <v>0</v>
       </c>
-      <c r="L8" s="60"/>
-      <c r="M8" s="61"/>
+      <c r="L8" s="61"/>
+      <c r="M8" s="62"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
@@ -2393,10 +2399,10 @@
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
       <c r="K10" s="50"/>
-      <c r="L10" s="73" t="s">
+      <c r="L10" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="M10" s="74"/>
+      <c r="M10" s="75"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
@@ -2405,19 +2411,19 @@
       <c r="B11" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="75" t="s">
+      <c r="C11" s="76" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="76"/>
-      <c r="E11" s="76"/>
-      <c r="F11" s="76"/>
-      <c r="G11" s="76"/>
-      <c r="H11" s="76"/>
-      <c r="I11" s="76"/>
-      <c r="J11" s="76"/>
-      <c r="K11" s="77"/>
-      <c r="L11" s="58"/>
-      <c r="M11" s="59"/>
+      <c r="D11" s="77"/>
+      <c r="E11" s="77"/>
+      <c r="F11" s="77"/>
+      <c r="G11" s="77"/>
+      <c r="H11" s="77"/>
+      <c r="I11" s="77"/>
+      <c r="J11" s="77"/>
+      <c r="K11" s="78"/>
+      <c r="L11" s="59"/>
+      <c r="M11" s="60"/>
     </row>
     <row r="12" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
@@ -2449,8 +2455,8 @@
       <c r="K12" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L12" s="58"/>
-      <c r="M12" s="59"/>
+      <c r="L12" s="59"/>
+      <c r="M12" s="60"/>
     </row>
     <row r="13" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
@@ -2469,8 +2475,8 @@
         <f>SUM(C13:J13)</f>
         <v>0</v>
       </c>
-      <c r="L13" s="58"/>
-      <c r="M13" s="59"/>
+      <c r="L13" s="59"/>
+      <c r="M13" s="60"/>
     </row>
     <row r="14" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
@@ -2489,25 +2495,25 @@
         <f>SUM(C14:J14)</f>
         <v>0</v>
       </c>
-      <c r="L14" s="58"/>
-      <c r="M14" s="59"/>
+      <c r="L14" s="59"/>
+      <c r="M14" s="60"/>
     </row>
     <row r="15" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
-      <c r="C15" s="78" t="s">
+      <c r="C15" s="79" t="s">
         <v>25</v>
       </c>
-      <c r="D15" s="79"/>
-      <c r="E15" s="79"/>
-      <c r="F15" s="79"/>
-      <c r="G15" s="79"/>
-      <c r="H15" s="79"/>
-      <c r="I15" s="79"/>
-      <c r="J15" s="79"/>
-      <c r="K15" s="80"/>
-      <c r="L15" s="58"/>
-      <c r="M15" s="59"/>
+      <c r="D15" s="80"/>
+      <c r="E15" s="80"/>
+      <c r="F15" s="80"/>
+      <c r="G15" s="80"/>
+      <c r="H15" s="80"/>
+      <c r="I15" s="80"/>
+      <c r="J15" s="80"/>
+      <c r="K15" s="81"/>
+      <c r="L15" s="59"/>
+      <c r="M15" s="60"/>
     </row>
     <row r="16" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
@@ -2539,8 +2545,8 @@
       <c r="K16" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="L16" s="58"/>
-      <c r="M16" s="59"/>
+      <c r="L16" s="59"/>
+      <c r="M16" s="60"/>
     </row>
     <row r="17" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
@@ -2559,8 +2565,8 @@
         <f>SUM(C17:J17)</f>
         <v>0</v>
       </c>
-      <c r="L17" s="58"/>
-      <c r="M17" s="59"/>
+      <c r="L17" s="59"/>
+      <c r="M17" s="60"/>
     </row>
     <row r="18" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="2"/>
@@ -2579,25 +2585,25 @@
         <f>SUM(C18:J18)</f>
         <v>0</v>
       </c>
-      <c r="L18" s="58"/>
-      <c r="M18" s="59"/>
+      <c r="L18" s="59"/>
+      <c r="M18" s="60"/>
     </row>
     <row r="19" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2"/>
       <c r="B19" s="4"/>
-      <c r="C19" s="81" t="s">
+      <c r="C19" s="82" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="79"/>
-      <c r="E19" s="79"/>
-      <c r="F19" s="79"/>
-      <c r="G19" s="79"/>
-      <c r="H19" s="79"/>
-      <c r="I19" s="79"/>
-      <c r="J19" s="79"/>
-      <c r="K19" s="80"/>
-      <c r="L19" s="58"/>
-      <c r="M19" s="59"/>
+      <c r="D19" s="80"/>
+      <c r="E19" s="80"/>
+      <c r="F19" s="80"/>
+      <c r="G19" s="80"/>
+      <c r="H19" s="80"/>
+      <c r="I19" s="80"/>
+      <c r="J19" s="80"/>
+      <c r="K19" s="81"/>
+      <c r="L19" s="59"/>
+      <c r="M19" s="60"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="2"/>
@@ -2629,8 +2635,8 @@
       <c r="K20" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="L20" s="58"/>
-      <c r="M20" s="59"/>
+      <c r="L20" s="59"/>
+      <c r="M20" s="60"/>
     </row>
     <row r="21" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2"/>
@@ -2649,8 +2655,8 @@
         <f>SUM(C21:J21)</f>
         <v>0</v>
       </c>
-      <c r="L21" s="58"/>
-      <c r="M21" s="59"/>
+      <c r="L21" s="59"/>
+      <c r="M21" s="60"/>
     </row>
     <row r="22" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2"/>
@@ -2669,8 +2675,8 @@
         <f>SUM(C22:J22)</f>
         <v>0</v>
       </c>
-      <c r="L22" s="58"/>
-      <c r="M22" s="59"/>
+      <c r="L22" s="59"/>
+      <c r="M22" s="60"/>
     </row>
     <row r="23" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="2"/>
@@ -2686,8 +2692,8 @@
       <c r="K23" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="L23" s="58"/>
-      <c r="M23" s="59"/>
+      <c r="L23" s="59"/>
+      <c r="M23" s="60"/>
     </row>
     <row r="24" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="2"/>
@@ -2704,15 +2710,15 @@
       <c r="F24" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="G24" s="82" t="s">
+      <c r="G24" s="83" t="s">
         <v>18</v>
       </c>
-      <c r="H24" s="83"/>
-      <c r="I24" s="83"/>
-      <c r="J24" s="84"/>
+      <c r="H24" s="84"/>
+      <c r="I24" s="84"/>
+      <c r="J24" s="85"/>
       <c r="K24" s="19"/>
-      <c r="L24" s="58"/>
-      <c r="M24" s="59"/>
+      <c r="L24" s="59"/>
+      <c r="M24" s="60"/>
     </row>
     <row r="25" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
@@ -2725,61 +2731,61 @@
       <c r="D25" s="11"/>
       <c r="E25" s="11"/>
       <c r="F25" s="11"/>
-      <c r="G25" s="69"/>
-      <c r="H25" s="70"/>
-      <c r="I25" s="70"/>
-      <c r="J25" s="71"/>
+      <c r="G25" s="70"/>
+      <c r="H25" s="71"/>
+      <c r="I25" s="71"/>
+      <c r="J25" s="72"/>
       <c r="K25" s="3">
         <f>SUM(C25:J25)</f>
         <v>0</v>
       </c>
-      <c r="L25" s="58"/>
-      <c r="M25" s="59"/>
+      <c r="L25" s="59"/>
+      <c r="M25" s="60"/>
     </row>
     <row r="26" spans="1:13" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="85" t="s">
+      <c r="A26" s="86" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="87" t="s">
+      <c r="B26" s="88" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="89" t="s">
+      <c r="C26" s="90" t="s">
         <v>31</v>
       </c>
-      <c r="D26" s="90"/>
-      <c r="E26" s="91" t="s">
+      <c r="D26" s="91"/>
+      <c r="E26" s="92" t="s">
         <v>32</v>
       </c>
-      <c r="F26" s="70"/>
-      <c r="G26" s="71"/>
-      <c r="H26" s="69" t="s">
+      <c r="F26" s="71"/>
+      <c r="G26" s="72"/>
+      <c r="H26" s="70" t="s">
         <v>33</v>
       </c>
-      <c r="I26" s="70"/>
-      <c r="J26" s="71"/>
+      <c r="I26" s="71"/>
+      <c r="J26" s="72"/>
       <c r="K26" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="L26" s="58"/>
-      <c r="M26" s="59"/>
+      <c r="L26" s="59"/>
+      <c r="M26" s="60"/>
     </row>
     <row r="27" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="86"/>
-      <c r="B27" s="88"/>
-      <c r="C27" s="92"/>
-      <c r="D27" s="93"/>
-      <c r="E27" s="91"/>
-      <c r="F27" s="70"/>
-      <c r="G27" s="72"/>
-      <c r="H27" s="89"/>
-      <c r="I27" s="94"/>
-      <c r="J27" s="90"/>
+      <c r="A27" s="87"/>
+      <c r="B27" s="89"/>
+      <c r="C27" s="93"/>
+      <c r="D27" s="94"/>
+      <c r="E27" s="92"/>
+      <c r="F27" s="71"/>
+      <c r="G27" s="73"/>
+      <c r="H27" s="90"/>
+      <c r="I27" s="95"/>
+      <c r="J27" s="91"/>
       <c r="K27" s="3">
         <f>SUM(C27:J27)</f>
         <v>0</v>
       </c>
-      <c r="L27" s="60"/>
-      <c r="M27" s="61"/>
+      <c r="L27" s="61"/>
+      <c r="M27" s="62"/>
     </row>
     <row r="28" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="12"/>
@@ -2826,10 +2832,10 @@
       <c r="K29" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="L29" s="73" t="s">
+      <c r="L29" s="74" t="s">
         <v>35</v>
       </c>
-      <c r="M29" s="74"/>
+      <c r="M29" s="75"/>
     </row>
     <row r="30" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
@@ -2847,8 +2853,8 @@
       <c r="I30" s="9"/>
       <c r="J30" s="9"/>
       <c r="K30" s="2"/>
-      <c r="L30" s="58"/>
-      <c r="M30" s="59"/>
+      <c r="L30" s="59"/>
+      <c r="M30" s="60"/>
     </row>
     <row r="31" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2"/>
@@ -2867,8 +2873,8 @@
         <f>SUM(C31:J31)</f>
         <v>0</v>
       </c>
-      <c r="L31" s="58"/>
-      <c r="M31" s="59"/>
+      <c r="L31" s="59"/>
+      <c r="M31" s="60"/>
     </row>
     <row r="32" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2"/>
@@ -2887,8 +2893,8 @@
         <f>SUM(C32:J32)</f>
         <v>0</v>
       </c>
-      <c r="L32" s="58"/>
-      <c r="M32" s="59"/>
+      <c r="L32" s="59"/>
+      <c r="M32" s="60"/>
     </row>
     <row r="33" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2"/>
@@ -2902,12 +2908,12 @@
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
       <c r="K33" s="9"/>
-      <c r="L33" s="58"/>
-      <c r="M33" s="59"/>
+      <c r="L33" s="59"/>
+      <c r="M33" s="60"/>
     </row>
     <row r="34" spans="1:13" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="95"/>
-      <c r="B34" s="97" t="s">
+      <c r="A34" s="96"/>
+      <c r="B34" s="98" t="s">
         <v>38</v>
       </c>
       <c r="C34" s="24" t="s">
@@ -2922,35 +2928,35 @@
       <c r="F34" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="G34" s="69" t="s">
+      <c r="G34" s="70" t="s">
         <v>18</v>
       </c>
-      <c r="H34" s="70"/>
-      <c r="I34" s="70"/>
-      <c r="J34" s="71"/>
+      <c r="H34" s="71"/>
+      <c r="I34" s="71"/>
+      <c r="J34" s="72"/>
       <c r="K34" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="L34" s="58"/>
-      <c r="M34" s="59"/>
+      <c r="L34" s="59"/>
+      <c r="M34" s="60"/>
     </row>
     <row r="35" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="96"/>
-      <c r="B35" s="98"/>
+      <c r="A35" s="97"/>
+      <c r="B35" s="99"/>
       <c r="C35" s="11"/>
       <c r="D35" s="11"/>
       <c r="E35" s="11"/>
       <c r="F35" s="11"/>
-      <c r="G35" s="69"/>
-      <c r="H35" s="70"/>
-      <c r="I35" s="70"/>
-      <c r="J35" s="72"/>
+      <c r="G35" s="70"/>
+      <c r="H35" s="71"/>
+      <c r="I35" s="71"/>
+      <c r="J35" s="73"/>
       <c r="K35" s="50">
         <f>SUM(C35:J35)</f>
         <v>0</v>
       </c>
-      <c r="L35" s="60"/>
-      <c r="M35" s="61"/>
+      <c r="L35" s="61"/>
+      <c r="M35" s="62"/>
     </row>
     <row r="36" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="25"/>
@@ -2997,10 +3003,10 @@
       <c r="K37" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="L37" s="99" t="s">
+      <c r="L37" s="100" t="s">
         <v>35</v>
       </c>
-      <c r="M37" s="74"/>
+      <c r="M37" s="75"/>
     </row>
     <row r="38" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
@@ -3018,8 +3024,8 @@
       <c r="I38" s="6"/>
       <c r="J38" s="6"/>
       <c r="K38" s="4"/>
-      <c r="L38" s="100"/>
-      <c r="M38" s="59"/>
+      <c r="L38" s="101"/>
+      <c r="M38" s="60"/>
     </row>
     <row r="39" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2"/>
@@ -3038,8 +3044,8 @@
         <f>SUM(C39:J39)</f>
         <v>0</v>
       </c>
-      <c r="L39" s="100"/>
-      <c r="M39" s="59"/>
+      <c r="L39" s="101"/>
+      <c r="M39" s="60"/>
     </row>
     <row r="40" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="2"/>
@@ -3058,8 +3064,8 @@
         <f>SUM(C40:J40)</f>
         <v>0</v>
       </c>
-      <c r="L40" s="100"/>
-      <c r="M40" s="59"/>
+      <c r="L40" s="101"/>
+      <c r="M40" s="60"/>
     </row>
     <row r="41" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2"/>
@@ -3073,12 +3079,12 @@
       <c r="I41" s="6"/>
       <c r="J41" s="6"/>
       <c r="K41" s="6"/>
-      <c r="L41" s="100"/>
-      <c r="M41" s="59"/>
+      <c r="L41" s="101"/>
+      <c r="M41" s="60"/>
     </row>
     <row r="42" spans="1:13" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="65"/>
-      <c r="B42" s="102" t="s">
+      <c r="A42" s="66"/>
+      <c r="B42" s="103" t="s">
         <v>41</v>
       </c>
       <c r="C42" s="11" t="s">
@@ -3093,35 +3099,35 @@
       <c r="F42" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="G42" s="69" t="s">
+      <c r="G42" s="70" t="s">
         <v>18</v>
       </c>
-      <c r="H42" s="70"/>
-      <c r="I42" s="70"/>
-      <c r="J42" s="71"/>
+      <c r="H42" s="71"/>
+      <c r="I42" s="71"/>
+      <c r="J42" s="72"/>
       <c r="K42" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="L42" s="100"/>
-      <c r="M42" s="59"/>
+      <c r="L42" s="101"/>
+      <c r="M42" s="60"/>
     </row>
     <row r="43" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="66"/>
-      <c r="B43" s="103"/>
+      <c r="A43" s="67"/>
+      <c r="B43" s="104"/>
       <c r="C43" s="21"/>
       <c r="D43" s="21"/>
       <c r="E43" s="21"/>
       <c r="F43" s="10"/>
-      <c r="G43" s="69"/>
-      <c r="H43" s="70"/>
-      <c r="I43" s="70"/>
-      <c r="J43" s="104"/>
+      <c r="G43" s="70"/>
+      <c r="H43" s="71"/>
+      <c r="I43" s="71"/>
+      <c r="J43" s="105"/>
       <c r="K43" s="22">
         <f>SUM(C43:J43)</f>
         <v>0</v>
       </c>
-      <c r="L43" s="101"/>
-      <c r="M43" s="61"/>
+      <c r="L43" s="102"/>
+      <c r="M43" s="62"/>
     </row>
     <row r="44" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="26"/>
@@ -3139,48 +3145,51 @@
       <c r="M44" s="26"/>
     </row>
     <row r="45" spans="1:13" ht="104.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="65" t="s">
+      <c r="A45" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="B45" s="109" t="s">
+      <c r="B45" s="110" t="s">
         <v>43</v>
       </c>
-      <c r="C45" s="105" t="s">
+      <c r="C45" s="106" t="s">
         <v>44</v>
       </c>
-      <c r="D45" s="106"/>
-      <c r="E45" s="107"/>
-      <c r="F45" s="108" t="s">
+      <c r="D45" s="107"/>
+      <c r="E45" s="108"/>
+      <c r="F45" s="109" t="s">
         <v>45</v>
       </c>
-      <c r="G45" s="70"/>
-      <c r="H45" s="104"/>
-      <c r="I45" s="108" t="s">
+      <c r="G45" s="71"/>
+      <c r="H45" s="105"/>
+      <c r="I45" s="109" t="s">
         <v>46</v>
       </c>
-      <c r="J45" s="71"/>
+      <c r="J45" s="72"/>
       <c r="K45" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="L45" s="73" t="s">
+      <c r="L45" s="74" t="s">
         <v>47</v>
       </c>
-      <c r="M45" s="74"/>
+      <c r="M45" s="75"/>
     </row>
     <row r="46" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="66"/>
-      <c r="B46" s="110"/>
-      <c r="C46" s="105"/>
-      <c r="D46" s="106"/>
-      <c r="E46" s="107"/>
-      <c r="F46" s="108"/>
-      <c r="G46" s="70"/>
-      <c r="H46" s="104"/>
-      <c r="I46" s="108"/>
-      <c r="J46" s="104"/>
-      <c r="K46" s="24"/>
-      <c r="L46" s="60"/>
-      <c r="M46" s="61"/>
+      <c r="A46" s="67"/>
+      <c r="B46" s="111"/>
+      <c r="C46" s="106"/>
+      <c r="D46" s="107"/>
+      <c r="E46" s="108"/>
+      <c r="F46" s="109"/>
+      <c r="G46" s="71"/>
+      <c r="H46" s="105"/>
+      <c r="I46" s="109"/>
+      <c r="J46" s="105"/>
+      <c r="K46" s="51">
+        <f>SUM(C46:J46)</f>
+        <v>0</v>
+      </c>
+      <c r="L46" s="61"/>
+      <c r="M46" s="62"/>
     </row>
     <row r="47" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="26"/>
@@ -3212,11 +3221,11 @@
       <c r="H48" s="9"/>
       <c r="I48" s="9"/>
       <c r="J48" s="9"/>
-      <c r="K48" s="2"/>
-      <c r="L48" s="73" t="s">
+      <c r="K48" s="50"/>
+      <c r="L48" s="74" t="s">
         <v>47</v>
       </c>
-      <c r="M48" s="111"/>
+      <c r="M48" s="112"/>
     </row>
     <row r="49" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
@@ -3233,9 +3242,9 @@
       <c r="H49" s="9"/>
       <c r="I49" s="9"/>
       <c r="J49" s="9"/>
-      <c r="K49" s="1"/>
-      <c r="L49" s="58"/>
-      <c r="M49" s="112"/>
+      <c r="K49" s="168"/>
+      <c r="L49" s="59"/>
+      <c r="M49" s="113"/>
     </row>
     <row r="50" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
@@ -3252,9 +3261,9 @@
       <c r="H50" s="9"/>
       <c r="I50" s="9"/>
       <c r="J50" s="9"/>
-      <c r="K50" s="1"/>
-      <c r="L50" s="60"/>
-      <c r="M50" s="113"/>
+      <c r="K50" s="168"/>
+      <c r="L50" s="61"/>
+      <c r="M50" s="114"/>
     </row>
     <row r="51" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
@@ -3271,11 +3280,11 @@
       <c r="H51" s="9"/>
       <c r="I51" s="9"/>
       <c r="J51" s="9"/>
-      <c r="K51" s="1"/>
-      <c r="L51" s="114" t="s">
+      <c r="K51" s="168"/>
+      <c r="L51" s="115" t="s">
         <v>56</v>
       </c>
-      <c r="M51" s="115"/>
+      <c r="M51" s="116"/>
     </row>
     <row r="52" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5"/>
@@ -3291,31 +3300,31 @@
       <c r="I52" s="5"/>
       <c r="J52" s="5"/>
       <c r="K52" s="5"/>
-      <c r="L52" s="116"/>
-      <c r="M52" s="117"/>
+      <c r="L52" s="117"/>
+      <c r="M52" s="118"/>
     </row>
     <row r="53" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2"/>
       <c r="B53" s="1"/>
-      <c r="C53" s="118" t="s">
+      <c r="C53" s="119" t="s">
         <v>11</v>
       </c>
-      <c r="D53" s="119"/>
-      <c r="E53" s="120"/>
-      <c r="F53" s="118" t="s">
+      <c r="D53" s="120"/>
+      <c r="E53" s="121"/>
+      <c r="F53" s="119" t="s">
         <v>12</v>
       </c>
-      <c r="G53" s="119"/>
-      <c r="H53" s="120"/>
+      <c r="G53" s="120"/>
+      <c r="H53" s="121"/>
       <c r="I53" s="9"/>
       <c r="J53" s="9"/>
       <c r="K53" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="L53" s="56" t="s">
+      <c r="L53" s="57" t="s">
         <v>58</v>
       </c>
-      <c r="M53" s="121"/>
+      <c r="M53" s="122"/>
     </row>
     <row r="54" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2"/>
@@ -3341,8 +3350,8 @@
       <c r="I54" s="9"/>
       <c r="J54" s="9"/>
       <c r="K54" s="1"/>
-      <c r="L54" s="58"/>
-      <c r="M54" s="112"/>
+      <c r="L54" s="59"/>
+      <c r="M54" s="113"/>
     </row>
     <row r="55" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
@@ -3360,8 +3369,8 @@
       <c r="I55" s="9"/>
       <c r="J55" s="9"/>
       <c r="K55" s="1"/>
-      <c r="L55" s="58"/>
-      <c r="M55" s="112"/>
+      <c r="L55" s="59"/>
+      <c r="M55" s="113"/>
     </row>
     <row r="56" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
@@ -3379,8 +3388,8 @@
       <c r="I56" s="9"/>
       <c r="J56" s="9"/>
       <c r="K56" s="1"/>
-      <c r="L56" s="58"/>
-      <c r="M56" s="112"/>
+      <c r="L56" s="59"/>
+      <c r="M56" s="113"/>
     </row>
     <row r="57" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
@@ -3398,8 +3407,8 @@
       <c r="I57" s="9"/>
       <c r="J57" s="9"/>
       <c r="K57" s="1"/>
-      <c r="L57" s="58"/>
-      <c r="M57" s="112"/>
+      <c r="L57" s="59"/>
+      <c r="M57" s="113"/>
     </row>
     <row r="58" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
@@ -3417,8 +3426,8 @@
       <c r="I58" s="9"/>
       <c r="J58" s="9"/>
       <c r="K58" s="1"/>
-      <c r="L58" s="58"/>
-      <c r="M58" s="112"/>
+      <c r="L58" s="59"/>
+      <c r="M58" s="113"/>
     </row>
     <row r="59" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
@@ -3436,8 +3445,8 @@
       <c r="I59" s="9"/>
       <c r="J59" s="9"/>
       <c r="K59" s="1"/>
-      <c r="L59" s="58"/>
-      <c r="M59" s="112"/>
+      <c r="L59" s="59"/>
+      <c r="M59" s="113"/>
     </row>
     <row r="60" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
@@ -3455,8 +3464,8 @@
       <c r="I60" s="9"/>
       <c r="J60" s="9"/>
       <c r="K60" s="1"/>
-      <c r="L60" s="58"/>
-      <c r="M60" s="112"/>
+      <c r="L60" s="59"/>
+      <c r="M60" s="113"/>
     </row>
     <row r="61" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A61" s="28"/>
@@ -3472,8 +3481,8 @@
       <c r="I61" s="28"/>
       <c r="J61" s="28"/>
       <c r="K61" s="30"/>
-      <c r="L61" s="58"/>
-      <c r="M61" s="112"/>
+      <c r="L61" s="59"/>
+      <c r="M61" s="113"/>
     </row>
     <row r="62" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A62" s="31" t="s">
@@ -3491,8 +3500,8 @@
       <c r="I62" s="9"/>
       <c r="J62" s="9"/>
       <c r="K62" s="2"/>
-      <c r="L62" s="58"/>
-      <c r="M62" s="112"/>
+      <c r="L62" s="59"/>
+      <c r="M62" s="113"/>
     </row>
     <row r="63" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A63" s="15" t="s">
@@ -3510,8 +3519,8 @@
       <c r="I63" s="9"/>
       <c r="J63" s="9"/>
       <c r="K63" s="2"/>
-      <c r="L63" s="58"/>
-      <c r="M63" s="112"/>
+      <c r="L63" s="59"/>
+      <c r="M63" s="113"/>
     </row>
     <row r="64" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A64" s="15" t="s">
@@ -3529,8 +3538,8 @@
       <c r="I64" s="9"/>
       <c r="J64" s="9"/>
       <c r="K64" s="2"/>
-      <c r="L64" s="58"/>
-      <c r="M64" s="112"/>
+      <c r="L64" s="59"/>
+      <c r="M64" s="113"/>
     </row>
     <row r="65" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="28"/>
@@ -3544,8 +3553,8 @@
       <c r="I65" s="28"/>
       <c r="J65" s="28"/>
       <c r="K65" s="28"/>
-      <c r="L65" s="58"/>
-      <c r="M65" s="112"/>
+      <c r="L65" s="59"/>
+      <c r="M65" s="113"/>
     </row>
     <row r="66" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
@@ -3563,8 +3572,8 @@
       <c r="I66" s="9"/>
       <c r="J66" s="9"/>
       <c r="K66" s="1"/>
-      <c r="L66" s="58"/>
-      <c r="M66" s="112"/>
+      <c r="L66" s="59"/>
+      <c r="M66" s="113"/>
     </row>
     <row r="67" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A67" s="33"/>
@@ -3580,8 +3589,8 @@
       <c r="I67" s="33"/>
       <c r="J67" s="33"/>
       <c r="K67" s="35"/>
-      <c r="L67" s="58"/>
-      <c r="M67" s="112"/>
+      <c r="L67" s="59"/>
+      <c r="M67" s="113"/>
     </row>
     <row r="68" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A68" s="31" t="s">
@@ -3599,8 +3608,8 @@
       <c r="I68" s="9"/>
       <c r="J68" s="9"/>
       <c r="K68" s="2"/>
-      <c r="L68" s="58"/>
-      <c r="M68" s="112"/>
+      <c r="L68" s="59"/>
+      <c r="M68" s="113"/>
     </row>
     <row r="69" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A69" s="15" t="s">
@@ -3618,8 +3627,8 @@
       <c r="I69" s="9"/>
       <c r="J69" s="9"/>
       <c r="K69" s="2"/>
-      <c r="L69" s="58"/>
-      <c r="M69" s="112"/>
+      <c r="L69" s="59"/>
+      <c r="M69" s="113"/>
     </row>
     <row r="70" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="15" t="s">
@@ -3637,8 +3646,8 @@
       <c r="I70" s="9"/>
       <c r="J70" s="9"/>
       <c r="K70" s="2"/>
-      <c r="L70" s="58"/>
-      <c r="M70" s="112"/>
+      <c r="L70" s="59"/>
+      <c r="M70" s="113"/>
     </row>
     <row r="71" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A71" s="28"/>
@@ -3652,8 +3661,8 @@
       <c r="I71" s="28"/>
       <c r="J71" s="28"/>
       <c r="K71" s="28"/>
-      <c r="L71" s="58"/>
-      <c r="M71" s="112"/>
+      <c r="L71" s="59"/>
+      <c r="M71" s="113"/>
     </row>
     <row r="72" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
@@ -3671,8 +3680,8 @@
       <c r="I72" s="9"/>
       <c r="J72" s="9"/>
       <c r="K72" s="2"/>
-      <c r="L72" s="58"/>
-      <c r="M72" s="112"/>
+      <c r="L72" s="59"/>
+      <c r="M72" s="113"/>
     </row>
     <row r="73" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="26"/>
@@ -3688,8 +3697,8 @@
       <c r="I73" s="26"/>
       <c r="J73" s="26"/>
       <c r="K73" s="37"/>
-      <c r="L73" s="58"/>
-      <c r="M73" s="112"/>
+      <c r="L73" s="59"/>
+      <c r="M73" s="113"/>
     </row>
     <row r="74" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="31" t="s">
@@ -3707,8 +3716,8 @@
       <c r="I74" s="9"/>
       <c r="J74" s="9"/>
       <c r="K74" s="2"/>
-      <c r="L74" s="58"/>
-      <c r="M74" s="112"/>
+      <c r="L74" s="59"/>
+      <c r="M74" s="113"/>
     </row>
     <row r="75" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A75" s="15" t="s">
@@ -3726,8 +3735,8 @@
       <c r="I75" s="9"/>
       <c r="J75" s="9"/>
       <c r="K75" s="2"/>
-      <c r="L75" s="58"/>
-      <c r="M75" s="112"/>
+      <c r="L75" s="59"/>
+      <c r="M75" s="113"/>
     </row>
     <row r="76" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="15" t="s">
@@ -3745,8 +3754,8 @@
       <c r="I76" s="9"/>
       <c r="J76" s="9"/>
       <c r="K76" s="2"/>
-      <c r="L76" s="122"/>
-      <c r="M76" s="123"/>
+      <c r="L76" s="123"/>
+      <c r="M76" s="124"/>
     </row>
     <row r="77" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="28"/>
@@ -3764,16 +3773,16 @@
       <c r="M77" s="30"/>
     </row>
     <row r="78" spans="1:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="124" t="s">
+      <c r="A78" s="125" t="s">
         <v>90</v>
       </c>
-      <c r="B78" s="125"/>
-      <c r="C78" s="125"/>
-      <c r="D78" s="125"/>
-      <c r="E78" s="125"/>
-      <c r="F78" s="125"/>
-      <c r="G78" s="125"/>
-      <c r="H78" s="126"/>
+      <c r="B78" s="126"/>
+      <c r="C78" s="126"/>
+      <c r="D78" s="126"/>
+      <c r="E78" s="126"/>
+      <c r="F78" s="126"/>
+      <c r="G78" s="126"/>
+      <c r="H78" s="127"/>
       <c r="I78" s="9"/>
       <c r="J78" s="9"/>
       <c r="K78" s="9"/>
@@ -3783,31 +3792,31 @@
     <row r="79" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2"/>
       <c r="B79" s="2"/>
-      <c r="C79" s="127" t="s">
+      <c r="C79" s="128" t="s">
         <v>11</v>
       </c>
-      <c r="D79" s="128"/>
-      <c r="E79" s="129"/>
-      <c r="F79" s="105" t="s">
+      <c r="D79" s="129"/>
+      <c r="E79" s="130"/>
+      <c r="F79" s="106" t="s">
         <v>12</v>
       </c>
-      <c r="G79" s="106"/>
-      <c r="H79" s="130"/>
+      <c r="G79" s="107"/>
+      <c r="H79" s="131"/>
       <c r="I79" s="9"/>
       <c r="J79" s="9"/>
       <c r="K79" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="L79" s="73" t="s">
+      <c r="L79" s="74" t="s">
         <v>91</v>
       </c>
-      <c r="M79" s="111"/>
+      <c r="M79" s="112"/>
     </row>
     <row r="80" spans="1:13" ht="68.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="65" t="s">
+      <c r="A80" s="66" t="s">
         <v>92</v>
       </c>
-      <c r="B80" s="131" t="s">
+      <c r="B80" s="132" t="s">
         <v>93</v>
       </c>
       <c r="C80" s="2" t="s">
@@ -3831,12 +3840,12 @@
       <c r="I80" s="9"/>
       <c r="J80" s="9"/>
       <c r="K80" s="5"/>
-      <c r="L80" s="58"/>
-      <c r="M80" s="112"/>
+      <c r="L80" s="59"/>
+      <c r="M80" s="113"/>
     </row>
     <row r="81" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="66"/>
-      <c r="B81" s="132"/>
+      <c r="A81" s="67"/>
+      <c r="B81" s="133"/>
       <c r="C81" s="1"/>
       <c r="D81" s="8"/>
       <c r="E81" s="8"/>
@@ -3846,8 +3855,8 @@
       <c r="I81" s="9"/>
       <c r="J81" s="9"/>
       <c r="K81" s="2"/>
-      <c r="L81" s="58"/>
-      <c r="M81" s="112"/>
+      <c r="L81" s="59"/>
+      <c r="M81" s="113"/>
     </row>
     <row r="82" spans="1:13" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
@@ -3865,8 +3874,8 @@
       <c r="I82" s="9"/>
       <c r="J82" s="9"/>
       <c r="K82" s="2"/>
-      <c r="L82" s="58"/>
-      <c r="M82" s="112"/>
+      <c r="L82" s="59"/>
+      <c r="M82" s="113"/>
     </row>
     <row r="83" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2"/>
@@ -3882,8 +3891,8 @@
       <c r="I83" s="9"/>
       <c r="J83" s="9"/>
       <c r="K83" s="4"/>
-      <c r="L83" s="58"/>
-      <c r="M83" s="112"/>
+      <c r="L83" s="59"/>
+      <c r="M83" s="113"/>
     </row>
     <row r="84" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2"/>
@@ -3899,8 +3908,8 @@
       <c r="I84" s="9"/>
       <c r="J84" s="9"/>
       <c r="K84" s="4"/>
-      <c r="L84" s="58"/>
-      <c r="M84" s="112"/>
+      <c r="L84" s="59"/>
+      <c r="M84" s="113"/>
     </row>
     <row r="85" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2"/>
@@ -3916,37 +3925,37 @@
       <c r="I85" s="9"/>
       <c r="J85" s="9"/>
       <c r="K85" s="4"/>
-      <c r="L85" s="122"/>
-      <c r="M85" s="123"/>
+      <c r="L85" s="123"/>
+      <c r="M85" s="124"/>
     </row>
     <row r="86" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A86" s="38"/>
       <c r="B86" s="38"/>
-      <c r="C86" s="133"/>
-      <c r="D86" s="134"/>
-      <c r="E86" s="134"/>
-      <c r="F86" s="134"/>
-      <c r="G86" s="134"/>
-      <c r="H86" s="134"/>
-      <c r="I86" s="134"/>
-      <c r="J86" s="134"/>
-      <c r="K86" s="135"/>
+      <c r="C86" s="134"/>
+      <c r="D86" s="135"/>
+      <c r="E86" s="135"/>
+      <c r="F86" s="135"/>
+      <c r="G86" s="135"/>
+      <c r="H86" s="135"/>
+      <c r="I86" s="135"/>
+      <c r="J86" s="135"/>
+      <c r="K86" s="136"/>
       <c r="L86" s="39"/>
       <c r="M86" s="39"/>
     </row>
     <row r="87" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="2"/>
       <c r="B87" s="2"/>
-      <c r="C87" s="127" t="s">
+      <c r="C87" s="128" t="s">
         <v>11</v>
       </c>
-      <c r="D87" s="128"/>
-      <c r="E87" s="129"/>
-      <c r="F87" s="69" t="s">
+      <c r="D87" s="129"/>
+      <c r="E87" s="130"/>
+      <c r="F87" s="70" t="s">
         <v>12</v>
       </c>
-      <c r="G87" s="70"/>
-      <c r="H87" s="71"/>
+      <c r="G87" s="71"/>
+      <c r="H87" s="72"/>
       <c r="I87" s="9"/>
       <c r="J87" s="17"/>
       <c r="K87" s="4" t="s">
@@ -3969,156 +3978,156 @@
       <c r="E88" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="F88" s="62"/>
+      <c r="F88" s="63"/>
       <c r="G88" s="40">
         <v>41913</v>
       </c>
       <c r="H88" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I88" s="138"/>
-      <c r="J88" s="141"/>
+      <c r="I88" s="139"/>
+      <c r="J88" s="142"/>
       <c r="K88" s="2"/>
-      <c r="L88" s="73" t="s">
+      <c r="L88" s="74" t="s">
         <v>91</v>
       </c>
-      <c r="M88" s="111"/>
+      <c r="M88" s="112"/>
     </row>
     <row r="89" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="2"/>
       <c r="B89" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="C89" s="157"/>
+      <c r="C89" s="158"/>
       <c r="D89" s="8"/>
       <c r="E89" s="8"/>
-      <c r="F89" s="136"/>
+      <c r="F89" s="137"/>
       <c r="G89" s="2"/>
       <c r="H89" s="8"/>
-      <c r="I89" s="139"/>
-      <c r="J89" s="142"/>
+      <c r="I89" s="140"/>
+      <c r="J89" s="143"/>
       <c r="K89" s="8"/>
-      <c r="L89" s="58"/>
-      <c r="M89" s="112"/>
+      <c r="L89" s="59"/>
+      <c r="M89" s="113"/>
     </row>
     <row r="90" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A90" s="2"/>
       <c r="B90" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C90" s="136"/>
+      <c r="C90" s="137"/>
       <c r="D90" s="1"/>
       <c r="E90" s="8"/>
-      <c r="F90" s="136"/>
+      <c r="F90" s="137"/>
       <c r="G90" s="8"/>
       <c r="H90" s="1"/>
-      <c r="I90" s="139"/>
-      <c r="J90" s="142"/>
+      <c r="I90" s="140"/>
+      <c r="J90" s="143"/>
       <c r="K90" s="8"/>
-      <c r="L90" s="58"/>
-      <c r="M90" s="112"/>
+      <c r="L90" s="59"/>
+      <c r="M90" s="113"/>
     </row>
     <row r="91" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2"/>
       <c r="B91" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C91" s="136"/>
+      <c r="C91" s="137"/>
       <c r="D91" s="1"/>
       <c r="E91" s="8"/>
-      <c r="F91" s="136"/>
+      <c r="F91" s="137"/>
       <c r="G91" s="8"/>
       <c r="H91" s="1"/>
-      <c r="I91" s="139"/>
-      <c r="J91" s="142"/>
+      <c r="I91" s="140"/>
+      <c r="J91" s="143"/>
       <c r="K91" s="8"/>
-      <c r="L91" s="58"/>
-      <c r="M91" s="112"/>
+      <c r="L91" s="59"/>
+      <c r="M91" s="113"/>
     </row>
     <row r="92" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2"/>
       <c r="B92" s="7" t="s">
         <v>104</v>
       </c>
-      <c r="C92" s="136"/>
+      <c r="C92" s="137"/>
       <c r="D92" s="1"/>
       <c r="E92" s="8"/>
-      <c r="F92" s="136"/>
+      <c r="F92" s="137"/>
       <c r="G92" s="8"/>
       <c r="H92" s="2"/>
-      <c r="I92" s="139"/>
-      <c r="J92" s="142"/>
+      <c r="I92" s="140"/>
+      <c r="J92" s="143"/>
       <c r="K92" s="1"/>
-      <c r="L92" s="58"/>
-      <c r="M92" s="112"/>
+      <c r="L92" s="59"/>
+      <c r="M92" s="113"/>
     </row>
     <row r="93" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2"/>
       <c r="B93" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C93" s="136"/>
+      <c r="C93" s="137"/>
       <c r="D93" s="1"/>
       <c r="E93" s="1"/>
-      <c r="F93" s="136"/>
+      <c r="F93" s="137"/>
       <c r="G93" s="1"/>
       <c r="H93" s="4"/>
-      <c r="I93" s="139"/>
-      <c r="J93" s="142"/>
+      <c r="I93" s="140"/>
+      <c r="J93" s="143"/>
       <c r="K93" s="1"/>
-      <c r="L93" s="58"/>
-      <c r="M93" s="112"/>
+      <c r="L93" s="59"/>
+      <c r="M93" s="113"/>
     </row>
     <row r="94" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2"/>
       <c r="B94" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C94" s="137"/>
+      <c r="C94" s="138"/>
       <c r="D94" s="1"/>
       <c r="E94" s="8"/>
-      <c r="F94" s="136"/>
+      <c r="F94" s="137"/>
       <c r="G94" s="8"/>
       <c r="H94" s="8"/>
-      <c r="I94" s="139"/>
-      <c r="J94" s="142"/>
+      <c r="I94" s="140"/>
+      <c r="J94" s="143"/>
       <c r="K94" s="8"/>
-      <c r="L94" s="58"/>
-      <c r="M94" s="112"/>
+      <c r="L94" s="59"/>
+      <c r="M94" s="113"/>
     </row>
     <row r="95" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A95" s="2"/>
       <c r="B95" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="C95" s="158"/>
+      <c r="C95" s="159"/>
       <c r="D95" s="8"/>
       <c r="E95" s="8"/>
-      <c r="F95" s="136"/>
+      <c r="F95" s="137"/>
       <c r="G95" s="8"/>
       <c r="H95" s="8"/>
-      <c r="I95" s="139"/>
-      <c r="J95" s="142"/>
+      <c r="I95" s="140"/>
+      <c r="J95" s="143"/>
       <c r="K95" s="8"/>
-      <c r="L95" s="58"/>
-      <c r="M95" s="112"/>
+      <c r="L95" s="59"/>
+      <c r="M95" s="113"/>
     </row>
     <row r="96" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2"/>
       <c r="B96" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="C96" s="159"/>
+      <c r="C96" s="160"/>
       <c r="D96" s="2"/>
       <c r="E96" s="1"/>
-      <c r="F96" s="137"/>
+      <c r="F96" s="138"/>
       <c r="G96" s="2"/>
       <c r="H96" s="4"/>
-      <c r="I96" s="140"/>
-      <c r="J96" s="143"/>
+      <c r="I96" s="141"/>
+      <c r="J96" s="144"/>
       <c r="K96" s="1"/>
-      <c r="L96" s="58"/>
-      <c r="M96" s="112"/>
+      <c r="L96" s="59"/>
+      <c r="M96" s="113"/>
     </row>
     <row r="97" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A97" s="28"/>
@@ -4132,8 +4141,8 @@
       <c r="I97" s="28"/>
       <c r="J97" s="28"/>
       <c r="K97" s="32"/>
-      <c r="L97" s="58"/>
-      <c r="M97" s="112"/>
+      <c r="L97" s="59"/>
+      <c r="M97" s="113"/>
     </row>
     <row r="98" spans="1:13" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
@@ -4159,42 +4168,42 @@
       <c r="I98" s="9"/>
       <c r="J98" s="9"/>
       <c r="K98" s="4"/>
-      <c r="L98" s="58"/>
-      <c r="M98" s="112"/>
+      <c r="L98" s="59"/>
+      <c r="M98" s="113"/>
     </row>
     <row r="99" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2"/>
       <c r="B99" s="7" t="s">
         <v>108</v>
       </c>
-      <c r="C99" s="149"/>
+      <c r="C99" s="150"/>
       <c r="D99" s="2"/>
       <c r="E99" s="2"/>
-      <c r="F99" s="148"/>
+      <c r="F99" s="149"/>
       <c r="G99" s="2"/>
       <c r="H99" s="4"/>
-      <c r="I99" s="138"/>
-      <c r="J99" s="148"/>
+      <c r="I99" s="139"/>
+      <c r="J99" s="149"/>
       <c r="K99" s="8"/>
-      <c r="L99" s="58"/>
-      <c r="M99" s="112"/>
+      <c r="L99" s="59"/>
+      <c r="M99" s="113"/>
     </row>
     <row r="100" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2"/>
       <c r="B100" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="C100" s="151"/>
+      <c r="C100" s="152"/>
       <c r="D100" s="2"/>
       <c r="E100" s="2"/>
-      <c r="F100" s="143"/>
+      <c r="F100" s="144"/>
       <c r="G100" s="1"/>
       <c r="H100" s="2"/>
-      <c r="I100" s="140"/>
-      <c r="J100" s="143"/>
+      <c r="I100" s="141"/>
+      <c r="J100" s="144"/>
       <c r="K100" s="1"/>
-      <c r="L100" s="58"/>
-      <c r="M100" s="112"/>
+      <c r="L100" s="59"/>
+      <c r="M100" s="113"/>
     </row>
     <row r="101" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A101" s="28"/>
@@ -4208,29 +4217,29 @@
       <c r="I101" s="28"/>
       <c r="J101" s="28"/>
       <c r="K101" s="28"/>
-      <c r="L101" s="58"/>
-      <c r="M101" s="112"/>
+      <c r="L101" s="59"/>
+      <c r="M101" s="113"/>
     </row>
     <row r="102" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A102" s="41"/>
       <c r="B102" s="4"/>
-      <c r="C102" s="105" t="s">
+      <c r="C102" s="106" t="s">
         <v>11</v>
       </c>
-      <c r="D102" s="106"/>
-      <c r="E102" s="130"/>
-      <c r="F102" s="69" t="s">
+      <c r="D102" s="107"/>
+      <c r="E102" s="131"/>
+      <c r="F102" s="70" t="s">
         <v>12</v>
       </c>
-      <c r="G102" s="70"/>
-      <c r="H102" s="71"/>
-      <c r="I102" s="149"/>
-      <c r="J102" s="152"/>
+      <c r="G102" s="71"/>
+      <c r="H102" s="72"/>
+      <c r="I102" s="150"/>
+      <c r="J102" s="153"/>
       <c r="K102" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="L102" s="58"/>
-      <c r="M102" s="112"/>
+      <c r="L102" s="59"/>
+      <c r="M102" s="113"/>
     </row>
     <row r="103" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
@@ -4257,11 +4266,11 @@
       <c r="H103" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I103" s="150"/>
-      <c r="J103" s="153"/>
+      <c r="I103" s="151"/>
+      <c r="J103" s="154"/>
       <c r="K103" s="2"/>
-      <c r="L103" s="58"/>
-      <c r="M103" s="112"/>
+      <c r="L103" s="59"/>
+      <c r="M103" s="113"/>
     </row>
     <row r="104" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A104" s="2"/>
@@ -4272,11 +4281,11 @@
       <c r="F104" s="8"/>
       <c r="G104" s="8"/>
       <c r="H104" s="8"/>
-      <c r="I104" s="151"/>
-      <c r="J104" s="154"/>
+      <c r="I104" s="152"/>
+      <c r="J104" s="155"/>
       <c r="K104" s="2"/>
-      <c r="L104" s="58"/>
-      <c r="M104" s="112"/>
+      <c r="L104" s="59"/>
+      <c r="M104" s="113"/>
     </row>
     <row r="105" spans="1:13" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A105" s="42"/>
@@ -4325,10 +4334,10 @@
       <c r="K106" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="L106" s="58" t="s">
+      <c r="L106" s="59" t="s">
         <v>91</v>
       </c>
-      <c r="M106" s="112"/>
+      <c r="M106" s="113"/>
     </row>
     <row r="107" spans="1:13" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
@@ -4337,73 +4346,73 @@
       <c r="B107" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="C107" s="160" t="s">
+      <c r="C107" s="161" t="s">
         <v>120</v>
       </c>
-      <c r="D107" s="161"/>
-      <c r="E107" s="161"/>
-      <c r="F107" s="161"/>
-      <c r="G107" s="162"/>
-      <c r="H107" s="160"/>
-      <c r="I107" s="161"/>
-      <c r="J107" s="162"/>
+      <c r="D107" s="162"/>
+      <c r="E107" s="162"/>
+      <c r="F107" s="162"/>
+      <c r="G107" s="163"/>
+      <c r="H107" s="161"/>
+      <c r="I107" s="162"/>
+      <c r="J107" s="163"/>
       <c r="K107" s="8"/>
-      <c r="L107" s="58"/>
-      <c r="M107" s="112"/>
+      <c r="L107" s="59"/>
+      <c r="M107" s="113"/>
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A108" s="131" t="s">
+      <c r="A108" s="132" t="s">
         <v>22</v>
       </c>
       <c r="B108" s="23" t="s">
         <v>121</v>
       </c>
-      <c r="C108" s="85"/>
-      <c r="D108" s="85"/>
-      <c r="E108" s="85"/>
-      <c r="F108" s="85"/>
-      <c r="G108" s="85"/>
-      <c r="H108" s="85"/>
-      <c r="I108" s="85"/>
-      <c r="J108" s="85"/>
-      <c r="K108" s="85"/>
-      <c r="L108" s="58"/>
-      <c r="M108" s="112"/>
+      <c r="C108" s="86"/>
+      <c r="D108" s="86"/>
+      <c r="E108" s="86"/>
+      <c r="F108" s="86"/>
+      <c r="G108" s="86"/>
+      <c r="H108" s="86"/>
+      <c r="I108" s="86"/>
+      <c r="J108" s="86"/>
+      <c r="K108" s="86"/>
+      <c r="L108" s="59"/>
+      <c r="M108" s="113"/>
     </row>
     <row r="109" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A109" s="155"/>
+      <c r="A109" s="156"/>
       <c r="B109" s="45"/>
-      <c r="C109" s="156"/>
-      <c r="D109" s="156"/>
-      <c r="E109" s="156"/>
-      <c r="F109" s="156"/>
-      <c r="G109" s="156"/>
-      <c r="H109" s="156"/>
-      <c r="I109" s="156"/>
-      <c r="J109" s="156"/>
-      <c r="K109" s="156"/>
-      <c r="L109" s="58"/>
-      <c r="M109" s="112"/>
+      <c r="C109" s="157"/>
+      <c r="D109" s="157"/>
+      <c r="E109" s="157"/>
+      <c r="F109" s="157"/>
+      <c r="G109" s="157"/>
+      <c r="H109" s="157"/>
+      <c r="I109" s="157"/>
+      <c r="J109" s="157"/>
+      <c r="K109" s="157"/>
+      <c r="L109" s="59"/>
+      <c r="M109" s="113"/>
     </row>
     <row r="110" spans="1:13" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="155"/>
+      <c r="A110" s="156"/>
       <c r="B110" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="C110" s="86"/>
-      <c r="D110" s="86"/>
-      <c r="E110" s="86"/>
-      <c r="F110" s="86"/>
-      <c r="G110" s="86"/>
-      <c r="H110" s="86"/>
-      <c r="I110" s="86"/>
-      <c r="J110" s="86"/>
-      <c r="K110" s="86"/>
-      <c r="L110" s="58"/>
-      <c r="M110" s="112"/>
+      <c r="C110" s="87"/>
+      <c r="D110" s="87"/>
+      <c r="E110" s="87"/>
+      <c r="F110" s="87"/>
+      <c r="G110" s="87"/>
+      <c r="H110" s="87"/>
+      <c r="I110" s="87"/>
+      <c r="J110" s="87"/>
+      <c r="K110" s="87"/>
+      <c r="L110" s="59"/>
+      <c r="M110" s="113"/>
     </row>
     <row r="111" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A111" s="155"/>
+      <c r="A111" s="156"/>
       <c r="B111" s="20" t="s">
         <v>123</v>
       </c>
@@ -4416,11 +4425,11 @@
       <c r="I111" s="8"/>
       <c r="J111" s="1"/>
       <c r="K111" s="1"/>
-      <c r="L111" s="58"/>
-      <c r="M111" s="112"/>
+      <c r="L111" s="59"/>
+      <c r="M111" s="113"/>
     </row>
     <row r="112" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A112" s="155"/>
+      <c r="A112" s="156"/>
       <c r="B112" s="15" t="s">
         <v>124</v>
       </c>
@@ -4433,11 +4442,11 @@
       <c r="I112" s="8"/>
       <c r="J112" s="1"/>
       <c r="K112" s="1"/>
-      <c r="L112" s="58"/>
-      <c r="M112" s="112"/>
+      <c r="L112" s="59"/>
+      <c r="M112" s="113"/>
     </row>
     <row r="113" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A113" s="132"/>
+      <c r="A113" s="133"/>
       <c r="B113" s="7" t="s">
         <v>125</v>
       </c>
@@ -4450,50 +4459,50 @@
       <c r="I113" s="8"/>
       <c r="J113" s="1"/>
       <c r="K113" s="1"/>
-      <c r="L113" s="58"/>
-      <c r="M113" s="112"/>
+      <c r="L113" s="59"/>
+      <c r="M113" s="113"/>
     </row>
     <row r="114" spans="1:13" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="65" t="s">
+      <c r="A114" s="66" t="s">
         <v>27</v>
       </c>
-      <c r="B114" s="144" t="s">
+      <c r="B114" s="145" t="s">
         <v>126</v>
       </c>
-      <c r="C114" s="146" t="s">
+      <c r="C114" s="147" t="s">
         <v>127</v>
       </c>
-      <c r="D114" s="147"/>
-      <c r="E114" s="164" t="s">
+      <c r="D114" s="148"/>
+      <c r="E114" s="165" t="s">
         <v>128</v>
       </c>
-      <c r="F114" s="165"/>
-      <c r="G114" s="147"/>
-      <c r="H114" s="164" t="s">
+      <c r="F114" s="166"/>
+      <c r="G114" s="148"/>
+      <c r="H114" s="165" t="s">
         <v>129</v>
       </c>
-      <c r="I114" s="165"/>
-      <c r="J114" s="166"/>
+      <c r="I114" s="166"/>
+      <c r="J114" s="167"/>
       <c r="K114" s="46" t="s">
         <v>6</v>
       </c>
-      <c r="L114" s="58"/>
-      <c r="M114" s="112"/>
+      <c r="L114" s="59"/>
+      <c r="M114" s="113"/>
     </row>
     <row r="115" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A115" s="66"/>
-      <c r="B115" s="145"/>
-      <c r="C115" s="91"/>
-      <c r="D115" s="104"/>
-      <c r="E115" s="108"/>
-      <c r="F115" s="70"/>
-      <c r="G115" s="104"/>
-      <c r="H115" s="108"/>
-      <c r="I115" s="70"/>
-      <c r="J115" s="71"/>
+      <c r="A115" s="67"/>
+      <c r="B115" s="146"/>
+      <c r="C115" s="92"/>
+      <c r="D115" s="105"/>
+      <c r="E115" s="109"/>
+      <c r="F115" s="71"/>
+      <c r="G115" s="105"/>
+      <c r="H115" s="109"/>
+      <c r="I115" s="71"/>
+      <c r="J115" s="72"/>
       <c r="K115" s="1"/>
-      <c r="L115" s="60"/>
-      <c r="M115" s="113"/>
+      <c r="L115" s="61"/>
+      <c r="M115" s="114"/>
     </row>
     <row r="116" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A116" s="28"/>
@@ -4540,10 +4549,10 @@
       <c r="K117" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="L117" s="73" t="s">
+      <c r="L117" s="74" t="s">
         <v>91</v>
       </c>
-      <c r="M117" s="111"/>
+      <c r="M117" s="112"/>
     </row>
     <row r="118" spans="1:13" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
@@ -4552,36 +4561,36 @@
       <c r="B118" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="C118" s="160" t="s">
+      <c r="C118" s="161" t="s">
         <v>132</v>
       </c>
-      <c r="D118" s="161"/>
-      <c r="E118" s="161"/>
-      <c r="F118" s="161"/>
-      <c r="G118" s="161"/>
-      <c r="H118" s="161"/>
-      <c r="I118" s="161"/>
-      <c r="J118" s="162"/>
+      <c r="D118" s="162"/>
+      <c r="E118" s="162"/>
+      <c r="F118" s="162"/>
+      <c r="G118" s="162"/>
+      <c r="H118" s="162"/>
+      <c r="I118" s="162"/>
+      <c r="J118" s="163"/>
       <c r="K118" s="8"/>
-      <c r="L118" s="58"/>
-      <c r="M118" s="112"/>
+      <c r="L118" s="59"/>
+      <c r="M118" s="113"/>
     </row>
     <row r="119" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A119" s="2"/>
       <c r="B119" s="47" t="s">
         <v>133</v>
       </c>
-      <c r="C119" s="163"/>
-      <c r="D119" s="56"/>
-      <c r="E119" s="56"/>
-      <c r="F119" s="56"/>
-      <c r="G119" s="56"/>
-      <c r="H119" s="56"/>
-      <c r="I119" s="56"/>
-      <c r="J119" s="56"/>
-      <c r="K119" s="121"/>
-      <c r="L119" s="58"/>
-      <c r="M119" s="112"/>
+      <c r="C119" s="164"/>
+      <c r="D119" s="57"/>
+      <c r="E119" s="57"/>
+      <c r="F119" s="57"/>
+      <c r="G119" s="57"/>
+      <c r="H119" s="57"/>
+      <c r="I119" s="57"/>
+      <c r="J119" s="57"/>
+      <c r="K119" s="122"/>
+      <c r="L119" s="59"/>
+      <c r="M119" s="113"/>
     </row>
     <row r="120" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2"/>
@@ -4597,8 +4606,8 @@
       <c r="I120" s="4"/>
       <c r="J120" s="1"/>
       <c r="K120" s="2"/>
-      <c r="L120" s="58"/>
-      <c r="M120" s="112"/>
+      <c r="L120" s="59"/>
+      <c r="M120" s="113"/>
     </row>
     <row r="121" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A121" s="2"/>
@@ -4614,8 +4623,8 @@
       <c r="I121" s="8"/>
       <c r="J121" s="1"/>
       <c r="K121" s="1"/>
-      <c r="L121" s="58"/>
-      <c r="M121" s="112"/>
+      <c r="L121" s="59"/>
+      <c r="M121" s="113"/>
     </row>
     <row r="122" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2"/>
@@ -4631,8 +4640,8 @@
       <c r="I122" s="8"/>
       <c r="J122" s="1"/>
       <c r="K122" s="1"/>
-      <c r="L122" s="60"/>
-      <c r="M122" s="113"/>
+      <c r="L122" s="61"/>
+      <c r="M122" s="114"/>
     </row>
   </sheetData>
   <mergeCells count="94">

</xml_diff>